<commit_message>
Add OSS/vendor classification column to report
各 JAR がオープンソース系か商用ベンダー系かを推定する「種別(OSS/ベンダー)」列を
Excel レポートに追加。

- classify_source_type(): ライセンス→groupId プレフィックス→ベンダー名の順で
  OSS / ベンダー系 / 要確認 を推定 (ライセンスが最優先の確定材料)
- JarReport.sourceType を追加し全行に付与
- 種別セルを色分け (OSS=緑 / ベンダー系=橙 / 要確認=灰) し、メタ情報行に
  OSS/ベンダー件数の集計を追記、凡例シートに判定基準を説明
- samples/make_demo_jars.py に商用ベンダー例 (Oracle ojdbc11) を追加し
  サンプル xlsx を再生成
- README のカラム一覧と説明を更新

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H7hCkxPxrsnvFKy7SmMucR
</commit_message>
<xml_diff>
--- a/samples/jars_report_sample.xlsx
+++ b/samples/jars_report_sample.xlsx
@@ -11,7 +11,7 @@
     <sheet name="凡例" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'JAR 一覧'!$A$3:$U$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'JAR 一覧'!$A$3:$V$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,11 @@
     </font>
     <font>
       <name val="Meiryo"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
       <color rgb="000563C1"/>
       <sz val="9"/>
       <u val="single"/>
@@ -62,7 +67,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -91,12 +96,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD9A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF1FB"/>
+        <fgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -126,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -146,38 +166,50 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -546,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -560,16 +592,17 @@
     <col width="46" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="60" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="44" customWidth="1" min="19" max="19"/>
-    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="44" customWidth="1" min="20" max="20"/>
     <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -582,7 +615,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>生成日時: 2026-07-08 05:31:23   |   走査対象: /tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo2   |   総数: 5 件   |   groupId 未確定: 1 件   |   推定補完: 3 件   |   モード: offline</t>
+          <t>生成日時: 2026-07-08 05:37:22   |   走査対象: /tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo3   |   総数: 6 件   |   OSS: 4 件 / ベンダー系: 1 件   |   groupId 未確定: 1 件   |   推定補完: 3 件   |   モード: offline</t>
         </is>
       </c>
     </row>
@@ -644,50 +677,55 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
+          <t>種別(OSS/ベンダー)</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
           <t>プロジェクト URL</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>座標の判定元</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>推定</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>取得 URL</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>取得元リポジトリ</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>URL 確認</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>サイズ</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>SHA-1</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>配置ディレクトリ</t>
         </is>
       </c>
-      <c r="U3" s="3" t="inlineStr">
+      <c r="V3" s="3" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
@@ -739,405 +777,521 @@
       </c>
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="6" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>OSS</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>既知マッピング</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>推定</t>
         </is>
       </c>
-      <c r="O4" s="7" t="inlineStr">
+      <c r="P4" s="8" t="inlineStr">
         <is>
           <t>https://repo1.maven.org/maven2/com/google/guava/guava/32.1.3/guava-32.1.3-jre.jar</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>Maven Central (候補)</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr">
         <is>
           <t>未確認 (offline)</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="S4" s="5" t="inlineStr">
         <is>
           <t>203 B</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
-        <is>
-          <t>901a4342e1368b2ad25d283aace84fc01f241e4b</t>
-        </is>
-      </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo2</t>
-        </is>
-      </c>
-      <c r="U4" s="6" t="inlineStr"/>
+          <t>7a2848b6c1901bb912d8e0510821480d8e3d1c3e</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo3</t>
+        </is>
+      </c>
+      <c r="V4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>ojdbc11-23.3.0.0.jar</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>com.oracle.database.jdbc</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>ojdbc11</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>23.3.0.0</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr"/>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>jar</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>JDBC</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr"/>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Oracle Corporation</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Oracle Free Use Terms and Conditions</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>ベンダー系</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr"/>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>pom.properties</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr"/>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t>https://repo1.maven.org/maven2/com/oracle/database/jdbc/ojdbc11/23.3.0.0/ojdbc11-23.3.0.0.jar</t>
+        </is>
+      </c>
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>Maven Central (候補)</t>
+        </is>
+      </c>
+      <c r="R5" s="10" t="inlineStr">
+        <is>
+          <t>未確認 (offline)</t>
+        </is>
+      </c>
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>531 B</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>a5e8c4c2d93637f5b9582fc49eb397eae849dc02</t>
+        </is>
+      </c>
+      <c r="U5" s="10" t="inlineStr">
+        <is>
+          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo3</t>
+        </is>
+      </c>
+      <c r="V5" s="11" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>commons-lang3.jar</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>org.apache.commons</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>commons-lang3</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>3.14.0</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>jar</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Apache Commons Lang</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Apache Commons Lang。java.lang を補完するユーティリティ群。</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>The Apache Software Foundation</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr"/>
-      <c r="L5" s="5" t="inlineStr"/>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>OSS</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>MANIFEST + 既知マッピング</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>推定</t>
         </is>
       </c>
-      <c r="O5" s="7" t="inlineStr">
+      <c r="P6" s="8" t="inlineStr">
         <is>
           <t>https://repo1.maven.org/maven2/org/apache/commons/commons-lang3/3.14.0/commons-lang3-3.14.0.jar</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr">
+      <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>Maven Central (候補)</t>
         </is>
       </c>
-      <c r="Q5" s="5" t="inlineStr">
+      <c r="R6" s="5" t="inlineStr">
         <is>
           <t>未確認 (offline)</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="S6" s="5" t="inlineStr">
         <is>
           <t>244 B</t>
         </is>
       </c>
-      <c r="S5" s="5" t="inlineStr">
-        <is>
-          <t>cfa448eb337939f79e87a15255a072dd058ead4f</t>
-        </is>
-      </c>
-      <c r="T5" s="5" t="inlineStr">
-        <is>
-          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo2</t>
-        </is>
-      </c>
-      <c r="U5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>2a1519c9274aa5db982a88cde71577ab0a4292b5</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo3</t>
+        </is>
+      </c>
+      <c r="V6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>log4j-core-2.22.1.jar</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>org.apache.logging.log4j</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>log4j-core</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>2.22.1</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr"/>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>jar</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>Apache Log4j Core</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>The Apache Log4j Implementation</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>The Apache Software Foundation</t>
         </is>
       </c>
-      <c r="K6" s="10" t="inlineStr">
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>Apache-2.0</t>
         </is>
       </c>
-      <c r="L6" s="11" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>OSS</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
         <is>
           <t>https://logging.apache.org/log4j/2.x/</t>
         </is>
       </c>
-      <c r="M6" s="10" t="inlineStr">
+      <c r="N7" s="11" t="inlineStr">
         <is>
           <t>pom.properties</t>
         </is>
       </c>
-      <c r="N6" s="8" t="inlineStr"/>
-      <c r="O6" s="11" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr"/>
+      <c r="P7" s="13" t="inlineStr">
         <is>
           <t>https://repo1.maven.org/maven2/org/apache/logging/log4j/log4j-core/2.22.1/log4j-core-2.22.1.jar</t>
         </is>
       </c>
-      <c r="P6" s="9" t="inlineStr">
+      <c r="Q7" s="10" t="inlineStr">
         <is>
           <t>Maven Central (候補)</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="inlineStr">
+      <c r="R7" s="10" t="inlineStr">
         <is>
           <t>未確認 (offline)</t>
         </is>
       </c>
-      <c r="R6" s="9" t="inlineStr">
+      <c r="S7" s="10" t="inlineStr">
         <is>
           <t>929 B</t>
         </is>
       </c>
-      <c r="S6" s="9" t="inlineStr">
-        <is>
-          <t>8d4f4c5c9e35a84e78d748dfdba534986bf4c7d4</t>
-        </is>
-      </c>
-      <c r="T6" s="9" t="inlineStr">
-        <is>
-          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo2</t>
-        </is>
-      </c>
-      <c r="U6" s="10" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="T7" s="10" t="inlineStr">
+        <is>
+          <t>ee8ca4c8ea3c88dbdfba467cbf618e4fe1e9ed54</t>
+        </is>
+      </c>
+      <c r="U7" s="10" t="inlineStr">
+        <is>
+          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo3</t>
+        </is>
+      </c>
+      <c r="V7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>slf4j-api-2.0.9.jar</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>org.slf4j</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>slf4j-api</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>2.0.9</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>jar</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>slf4j-api</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>The slf4j API</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>QOS.ch</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>OSS</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr"/>
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>既知マッピング</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>推定</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr">
+      <c r="P8" s="8" t="inlineStr">
         <is>
           <t>https://repo1.maven.org/maven2/org/slf4j/slf4j-api/2.0.9/slf4j-api-2.0.9.jar</t>
         </is>
       </c>
-      <c r="P7" s="5" t="inlineStr">
+      <c r="Q8" s="5" t="inlineStr">
         <is>
           <t>Maven Central (候補)</t>
         </is>
       </c>
-      <c r="Q7" s="5" t="inlineStr">
+      <c r="R8" s="5" t="inlineStr">
         <is>
           <t>未確認 (offline)</t>
         </is>
       </c>
-      <c r="R7" s="5" t="inlineStr">
+      <c r="S8" s="5" t="inlineStr">
         <is>
           <t>244 B</t>
         </is>
       </c>
-      <c r="S7" s="5" t="inlineStr">
-        <is>
-          <t>3e6ce52a3e20487342e5fbdc766547e657303e3a</t>
-        </is>
-      </c>
-      <c r="T7" s="5" t="inlineStr">
-        <is>
-          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo2</t>
-        </is>
-      </c>
-      <c r="U7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>9278ba836275b6d01f5b9293448e72ae8e2bf227</t>
+        </is>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo3</t>
+        </is>
+      </c>
+      <c r="V8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>mystery-lib-1.0.jar</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>mystery-lib</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr"/>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>jar</t>
         </is>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>mystery-lib</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr"/>
-      <c r="J8" s="14" t="inlineStr"/>
-      <c r="K8" s="14" t="inlineStr"/>
-      <c r="L8" s="13" t="inlineStr"/>
-      <c r="M8" s="14" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr"/>
+      <c r="J9" s="16" t="inlineStr"/>
+      <c r="K9" s="16" t="inlineStr"/>
+      <c r="L9" s="17" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="M9" s="15" t="inlineStr"/>
+      <c r="N9" s="16" t="inlineStr">
         <is>
           <t>ファイル名推定</t>
         </is>
       </c>
-      <c r="N8" s="12" t="inlineStr"/>
-      <c r="O8" s="13" t="inlineStr"/>
-      <c r="P8" s="13" t="inlineStr"/>
-      <c r="Q8" s="13" t="inlineStr">
+      <c r="O9" s="14" t="inlineStr"/>
+      <c r="P9" s="15" t="inlineStr"/>
+      <c r="Q9" s="15" t="inlineStr"/>
+      <c r="R9" s="15" t="inlineStr">
         <is>
           <t>座標未確定のため生成不可</t>
         </is>
       </c>
-      <c r="R8" s="13" t="inlineStr">
+      <c r="S9" s="15" t="inlineStr">
         <is>
           <t>163 B</t>
         </is>
       </c>
-      <c r="S8" s="13" t="inlineStr">
-        <is>
-          <t>d9e89be65ea302797f91a5cb1aec235b40a1cd76</t>
-        </is>
-      </c>
-      <c r="T8" s="13" t="inlineStr">
-        <is>
-          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo2</t>
-        </is>
-      </c>
-      <c r="U8" s="14" t="inlineStr">
+      <c r="T9" s="15" t="inlineStr">
+        <is>
+          <t>1ae29a2625076aa35df4448ca0f6c17e46df91ee</t>
+        </is>
+      </c>
+      <c r="U9" s="15" t="inlineStr">
+        <is>
+          <t>/tmp/claude-0/-home-user-Jar-Downloader/13089bda-d5d0-54a2-b55d-ff5dceebdc84/scratchpad/demo3</t>
+        </is>
+      </c>
+      <c r="V9" s="16" t="inlineStr">
         <is>
           <t>groupId を特定できず。手動補正を推奨。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:U8"/>
+  <autoFilter ref="A3:V9"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1149,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1157,151 +1311,187 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>凡例・カラム説明</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>行の色</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>意味</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr"/>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr"/>
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>groupId を特定できなかった行 (要手動補正)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr"/>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr"/>
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>座標の一部をファイル名/マッピング/照合で推定・補完した行</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr"/>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr"/>
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>通常行 (交互の縞模様)</t>
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr"/>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>種別セル: OSS (オープンソース)</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr"/>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>種別セル: ベンダー系 (商用/独自ライセンス)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr"/>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>種別セル: 要確認 (判定材料が不足)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>カラム</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>説明</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>groupId / artifactId / version</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>Maven 座標。pom.properties→pom.xml→MANIFEST→既知マッピング→Maven Central 照合→ファイル名推定 の順に解決。</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>classifier</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>sources / javadoc 等の分類子 (ファイル名から推定)。</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>ライブラリ名 / 概要</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>pom.xml の name/description、MANIFEST、内蔵説明から構築。</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>種別(OSS/ベンダー)</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>提供形態の推定。ライセンス→groupId→ベンダー名の順で判定。OSS=オープンソース、ベンダー系=商用/独自ライセンス、要確認=判定不能。確定にはライセンス条項の確認を推奨。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>座標の判定元</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>どの情報源で座標を決定したか。'ファイル名推定' は最も不確実。</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>推定</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>座標の一部を推測で補った場合に '推定' と表示。</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>取得 URL</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>Maven 標準レイアウトで生成した取得先。online 時は実在確認済み。</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>URL 確認</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>online: 実在確認 OK / 全リポジトリで未検出、offline: 未確認、座標未確定時: 生成不可。</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>SHA-1</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>ファイルの SHA-1。--online の Maven Central 照合キーにも使用。</t>
         </is>

</xml_diff>